<commit_message>
Aplicación completa: frontend React, vistas de API, flujo de cambio y despliegue
- Frontend nuevo con las 12 pantallas (3 roles): proyectos, importación,
  actividades y precedencias, Carta Gantt SVG, recursos y costos, hitos,
  KPI, solicitudes de cambio (10 etapas), tableros, usuarios y caso de prueba.
- API de vistas /api/v1 (gantt, recursos, hitos, KPI, cambio, tableros).
- Corrige recálculo: la consolidación de costos usaba fechas obsoletas.
- Imagen Docker única, docker-compose, render.yaml y scripts .bat.
- Pruebas de integración con PostgreSQL de los 3 escenarios de la demo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011HCEms5rULWvVeWhJXC4TD
</commit_message>
<xml_diff>
--- a/seeds/Seed_B_Caso_Prueba_Minimo.xlsx
+++ b/seeds/Seed_B_Caso_Prueba_Minimo.xlsx
@@ -41,7 +41,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SEED-B-MINIMO</t>
+          <t>CASO-PRUEBA</t>
         </is>
       </c>
     </row>
@@ -53,7 +53,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Caso de prueba mínimo</t>
+          <t>Caso de prueba mínimo · App de inspecciones</t>
         </is>
       </c>
     </row>
@@ -77,7 +77,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
@@ -89,7 +89,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
@@ -101,7 +101,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2027-01-29</t>
         </is>
       </c>
     </row>
@@ -113,7 +113,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>45000000</t>
+          <t>30287400</t>
         </is>
       </c>
     </row>
@@ -161,7 +161,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -195,19 +195,49 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>meta</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>adicional</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SPI</t>
+          <t>P01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Índice de desempeño de plazo</t>
+          <t>Índice de desempeño del cronograma (SPI)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -222,19 +252,44 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>índice</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Valor ganado sobre valor planificado a la fecha de corte.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CPI</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Índice de desempeño de costo</t>
+          <t>Índice de desempeño de costo (CPI)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -249,19 +304,44 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>índice</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Valor ganado sobre costo real a la fecha de corte.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Variación de plazo</t>
+          <t>Variación del cronograma (SV)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -276,19 +356,44 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-2000000</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CLP</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Diferencia entre valor ganado y valor planificado.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Variación de costo</t>
+          <t>Variación de costo (CV)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -303,14 +408,39 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-2000000</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CLP</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Diferencia entre valor ganado y costo real.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADVANCE_GAP</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -320,7 +450,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>avance_real - avance_plan</t>
+          <t>AVANCE_REAL - AVANCE_PLAN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -330,14 +460,39 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Avance real menos avance planificado, en puntos porcentuales.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LATE_TASKS</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -347,7 +502,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>count(actividades_atrasadas) / count(actividades)</t>
+          <t>count(ACTIVIDADES_ATRASADAS) / count(ACTIVIDADES) * 100</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -357,14 +512,39 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Subactividades iniciadas o vencidas con avance bajo lo planificado.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MILESTONE_ON_TIME</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -374,7 +554,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>count(hitos_a_tiempo) / count(hitos)</t>
+          <t>MILESTONES_ON_TIME_PCT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -384,14 +564,39 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Hitos cumplidos en o antes de su fecha base, sobre hitos cumplidos.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLOSE_VARIANCE</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -401,7 +606,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>fecha_cierre_real - fecha_cierre_base</t>
+          <t>CLOSING_MILESTONE_DEVIATION</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -411,7 +616,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PROYECTO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Días hábiles entre la fecha proyectada y la fecha base del cierre.</t>
         </is>
       </c>
     </row>
@@ -445,24 +675,54 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>meta</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>unidad</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>adicional</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CHG-01</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>solicitudes registradas</t>
+          <t>Solicitudes registradas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>valor_01</t>
+          <t>CHANGE_REQUESTS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -472,24 +732,34 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>n°</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Total de solicitudes de cambio del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CHG-02</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tasa de aprobación</t>
+          <t>Tasa de aprobación</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>valor_02</t>
+          <t>CHANGE_APPROVAL_RATE * 100</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -499,24 +769,34 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Aprobadas sobre decididas.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CHG-03</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tasa de rechazo</t>
+          <t>Tasa de rechazo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>valor_03</t>
+          <t>CHANGE_REJECTION_RATE * 100</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -526,24 +806,34 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Rechazadas sobre decididas.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHG-04</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tiempo medio de ciclo</t>
+          <t>Tiempo medio de ciclo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>valor_04</t>
+          <t>CHANGE_AVG_CYCLE_HOURS / 24</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -553,24 +843,49 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Promedio de días entre registro y cierre de las solicitudes cerradas.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHG-05</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tiempo medio de evaluación de impacto</t>
+          <t>Tiempo medio de evaluación de impacto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>valor_05</t>
+          <t>CHANGE_AVG_IMPACT_HOURS / 24</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -580,24 +895,49 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Promedio de días entre registro y primer análisis de impacto.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CHG-06</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>impacto acumulado en costo</t>
+          <t>Impacto acumulado en costo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>valor_06</t>
+          <t>CHANGE_IMPACT_COST</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -607,24 +947,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>CLP</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Suma del delta de costo de los cambios aprobados.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CHG-07</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>impacto acumulado en plazo</t>
+          <t>Impacto acumulado en plazo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>valor_07</t>
+          <t>CHANGE_IMPACT_DAYS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -634,24 +984,49 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Suma del delta de plazo de los cambios aprobados.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CHG-08</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>% con evidencia completa</t>
+          <t>Solicitudes con evidencia completa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>valor_08</t>
+          <t>CHANGE_EVIDENCE_COMPLETE_PCT * 100</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -661,24 +1036,49 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Solicitudes con al menos una evidencia sobre el total.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CHG-09</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>solicitudes fuera de SLA</t>
+          <t>Solicitudes fuera de SLA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>valor_09</t>
+          <t>CHANGE_SLA_BREACHES</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -688,24 +1088,49 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>n°</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Solicitudes abiertas cuya etapa activa superó su SLA.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHG-10</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>consumo de contingencia</t>
+          <t>Consumo de contingencia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>valor_10</t>
+          <t>CHANGE_CONTINGENCY_CONSUMPTION</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -715,24 +1140,54 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Costo de cambios aprobados sobre la contingencia del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CHG-11</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>índice de adopción</t>
+          <t>Índice de adopción</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>valor_11</t>
+          <t>CHANGE_ADOPTION_INDEX</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -742,24 +1197,54 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Usuarios activos sobre usuarios capacitados (variable manual).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CHG-12</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>cobertura de capacitación</t>
+          <t>Cobertura de capacitación</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>valor_12</t>
+          <t>CHANGE_TRAINING_COVERAGE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -769,7 +1254,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>CAMBIO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Usuarios capacitados sobre usuarios objetivo (variable manual).</t>
         </is>
       </c>
     </row>
@@ -820,14 +1335,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>['SPI', 'CPI', 'SV', 'CV', 'ADVANCE_GAP', 'LATE_TASKS', 'MILESTONE_ON_TIME', 'CLOSE_VARIANCE']</t>
+          <t>P01,P02,P03,P04,P05,P06,P07,P08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DB-CAMBIOS</t>
+          <t>DB-CAMBIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -842,7 +1357,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>['CHG-01', 'CHG-02', 'CHG-03', 'CHG-04', 'CHG-05', 'CHG-06', 'CHG-07', 'CHG-08', 'CHG-09', 'CHG-10', 'CHG-11', 'CHG-12']</t>
+          <t>C01,C02,C03,C04,C05,C06,C07,C08,C09,C10,C11,C12</t>
         </is>
       </c>
     </row>
@@ -877,7 +1392,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2026-05-01</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -886,7 +1401,142 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Día del Trabajo</t>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2026-10-12</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026-10-31</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026-11-01</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2026-12-08</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2026-12-25</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2027-01-01</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2027-03-26</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2027-03-27</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FERIADO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Feriado nacional</t>
         </is>
       </c>
     </row>
@@ -962,7 +1612,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -972,109 +1622,215 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Inicio y definición</t>
+          <t>Inicio y requisitos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>AC1.1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ETAPA</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Diseño y construcción</t>
+          <t>Inicio del proyecto</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>E1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ETAPA</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Integración y pruebas</t>
+          <t>Realizar kick-off y plan de trabajo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AC1.1</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2026-09-07</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2026-09-09</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>2026-09-07</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2026-09-09</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>984000</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>AC1.2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ETAPA</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Despliegue y cierre</t>
+          <t>Levantamiento en obra</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>E1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Alineamiento inicial</t>
+          <t>Entrevistar a jefes de obra e inspectores</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>AC1.2</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2026-09-10</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2026-09-16</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>A01FS</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>2026-09-10</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2026-09-16</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>968000</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Requisitos</t>
+          <t>Redactar historias de usuario</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>AC1.2</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2026-09-14</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>A02SS+2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>2026-09-14</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2026-09-22</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>888000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC1.3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1084,85 +1840,139 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Plan de trabajo</t>
+          <t>Alcance y backlog</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>E1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AC21</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Diseño funcional</t>
+          <t>Priorizar backlog con el cliente</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>AC1.3</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2026-09-23</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2026-09-24</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>A03FS</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>2026-09-23</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2026-09-24</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>416000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AC22</t>
+          <t>H01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>HITO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Construcción núcleo</t>
+          <t>Alcance aprobado</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E02</t>
-        </is>
+          <t>AC1.3</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2026-09-24</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2026-09-24</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>A04FS</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>2026-09-24</v>
+      </c>
+      <c r="K10" t="n">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AC23</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>ETAPA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Construcción móvil</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>E02</t>
+          <t>Diseño y construcción</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AC31</t>
+          <t>AC2.1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1172,85 +1982,176 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Integraciones</t>
+          <t>Diseño de la solución</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AC32</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pruebas técnicas</t>
+          <t>Diseñar prototipo UX de inspección</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>AC2.1</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2026-09-25</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2026-10-06</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>H01FS</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>2026-09-25</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2026-09-30</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1729600</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AC33</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Aceptación usuaria</t>
+          <t>Diseñar arquitectura y modelo de datos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>AC2.1</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2026-09-28</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2026-10-05</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>A05SS+1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2026-09-28</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2026-10-05</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>820800</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AC41</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>HITO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Preparación productiva</t>
+          <t>Diseño de solución aprobado</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>E04</t>
-        </is>
+          <t>AC2.1</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2026-10-06</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2026-10-06</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>A05FS;A06FS</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>2026-10-06</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2026-10-06</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AC42</t>
+          <t>AC2.2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1260,41 +2161,73 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Adopción</t>
+          <t>Construcción backend</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AC43</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ACTIVIDAD</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cierre</t>
+          <t>Construir API de inspecciones</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>AC2.2</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2026-10-07</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>H02FS</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>2026-10-07</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2026-10-21</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>3620000</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1304,78 +2237,73 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 01</t>
+          <t>Construir reportes y exportación</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC2.2</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2026-01-05</v>
+        <v>2026-10-22</v>
       </c>
       <c r="F18" t="n">
-        <v>2026-01-07</v>
+        <v>2026-10-29</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>A07FS</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>2026-10-22</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2026-10-29</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1152000</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>AC2.3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 02</t>
+          <t>Construcción app móvil</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>AC11</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>2026-01-08</v>
-      </c>
-      <c r="F19" t="n">
-        <v>2026-01-13</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>A01FS</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1385,40 +2313,48 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 03</t>
+          <t>Construir app móvil offline</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC2.3</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2026-01-14</v>
+        <v>2026-10-09</v>
       </c>
       <c r="F20" t="n">
-        <v>2026-01-20</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>A02SS</t>
+          <t>A07SS+2</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>2026-10-09</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1612800</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1428,71 +2364,79 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 04</t>
+          <t>Integrar captura de fotos georreferenciadas</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC2.3</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2026-01-21</v>
+        <v>2026-10-21</v>
       </c>
       <c r="F21" t="n">
-        <v>2026-01-23</v>
+        <v>2026-10-27</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>A03FF</t>
+          <t>A09FF</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>2026-10-21</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>192000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>HITO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 05</t>
+          <t>Release candidata lista</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>AC13</t>
+          <t>AC2.3</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2026-01-26</v>
+        <v>2026-10-29</v>
       </c>
       <c r="F22" t="n">
-        <v>2026-01-29</v>
+        <v>2026-10-29</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>A04SF</t>
+          <t>A08FS;A10FS</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1504,93 +2448,46 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ETAPA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 06</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>AC21</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>2026-01-30</v>
-      </c>
-      <c r="F23" t="n">
-        <v>2026-02-05</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>A05FS</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>Integración y pruebas</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>AC3.1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 07</t>
+          <t>Integraciones</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AC21</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>2026-02-06</v>
-      </c>
-      <c r="F24" t="n">
-        <v>2026-02-10</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>A06FS</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1600,19 +2497,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 08</t>
+          <t>Integrar inicio de sesión corporativo (SSO)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AC22</t>
+          <t>AC3.1</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2026-02-11</v>
+        <v>2026-10-30</v>
       </c>
       <c r="F25" t="n">
-        <v>2026-02-16</v>
+        <v>2026-11-04</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1621,7 +2518,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>A07SS</t>
+          <t>H03FS</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1633,7 +2530,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1643,28 +2540,28 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 09</t>
+          <t>Integrar ERP en modo lectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AC22</t>
+          <t>AC3.1</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2026-02-17</v>
+        <v>2026-11-05</v>
       </c>
       <c r="F26" t="n">
-        <v>2026-02-23</v>
+        <v>2026-11-12</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>A08FS</t>
+          <t>A11FS</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1676,50 +2573,29 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>AC3.2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 10</t>
+          <t>Pruebas técnicas</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AC23</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>2026-02-24</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2026-02-26</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>A09FF</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1729,28 +2605,28 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 11</t>
+          <t>Ejecutar pruebas de sistema</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AC31</t>
+          <t>AC3.2</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>2026-02-27</v>
+        <v>2026-11-13</v>
       </c>
       <c r="F28" t="n">
-        <v>2026-03-04</v>
+        <v>2026-11-20</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>A10SF</t>
+          <t>A12FS</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1762,7 +2638,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1772,28 +2648,28 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 12</t>
+          <t>Ejecutar prueba de seguridad externa</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AC31</t>
+          <t>AC3.2</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2026-03-05</v>
+        <v>2026-11-18</v>
       </c>
       <c r="F29" t="n">
-        <v>2026-03-11</v>
+        <v>2026-11-20</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>A11FS</t>
+          <t>A13SS+3</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1805,50 +2681,29 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>AC3.3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 13</t>
+          <t>Aceptación usuaria</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AC32</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>2026-03-12</v>
-      </c>
-      <c r="F30" t="n">
-        <v>2026-03-16</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>A12FS</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E3</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>A15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1858,19 +2713,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 14</t>
+          <t>Realizar UAT con jefes de obra</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>AC32</t>
+          <t>AC3.3</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2026-03-17</v>
+        <v>2026-11-23</v>
       </c>
       <c r="F31" t="n">
-        <v>2026-03-20</v>
+        <v>2026-11-26</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1879,7 +2734,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>A13SS</t>
+          <t>A13FS;A14FS</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1891,38 +2746,38 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>H04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>HITO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 15</t>
+          <t>UAT aprobada</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AC33</t>
+          <t>AC3.3</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2026-03-23</v>
+        <v>2026-11-26</v>
       </c>
       <c r="F32" t="n">
-        <v>2026-03-27</v>
+        <v>2026-11-26</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>A14FS</t>
+          <t>A15FS</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1934,93 +2789,46 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>A16</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ETAPA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 16</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>AC41</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>2026-03-30</v>
-      </c>
-      <c r="F33" t="n">
-        <v>2026-04-01</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>A15FF</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>Despliegue y cierre</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>A17</t>
+          <t>AC4.1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 17</t>
+          <t>Preparación de usuarios</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>AC41</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>2026-04-02</v>
-      </c>
-      <c r="F34" t="n">
-        <v>2026-04-07</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>A16FS</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>A18</t>
+          <t>A16</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2030,28 +2838,28 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 18</t>
+          <t>Capacitar a usuarios de obra</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AC42</t>
+          <t>AC4.1</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>2026-04-08</v>
+        <v>2026-11-24</v>
       </c>
       <c r="F35" t="n">
-        <v>2026-04-14</v>
+        <v>2026-11-27</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>A17SF</t>
+          <t>A15SS+1;A17SF</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2063,50 +2871,29 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>A19</t>
+          <t>AC4.2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SUBACTIVIDAD</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 19</t>
+          <t>Puesta en marcha</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>AC42</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>2026-04-15</v>
-      </c>
-      <c r="F36" t="n">
-        <v>2026-04-17</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>A18FS</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E4</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>A20</t>
+          <t>A17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2116,28 +2903,28 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Trabajo demostrable 20</t>
+          <t>Desplegar en producción</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>AC43</t>
+          <t>AC4.2</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>2026-04-20</v>
+        <v>2026-11-27</v>
       </c>
       <c r="F37" t="n">
-        <v>2026-04-23</v>
+        <v>2026-11-27</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>A19FS</t>
+          <t>H04FS</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2149,7 +2936,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>H01</t>
+          <t>H05</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2159,19 +2946,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Acta de inicio aprobada</t>
+          <t>Piloto en operación</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>AC11</t>
+          <t>AC4.2</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>2026-01-13</v>
+        <v>2026-11-27</v>
       </c>
       <c r="F38" t="n">
-        <v>2026-01-13</v>
+        <v>2026-11-27</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2180,7 +2967,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>A02FS</t>
+          <t>A17FS</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2192,38 +2979,38 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>H02</t>
+          <t>A18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HITO</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Requisitos validados</t>
+          <t>Acompañar operación asistida</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>AC12</t>
+          <t>AC4.2</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2026-01-23</v>
+        <v>2026-11-30</v>
       </c>
       <c r="F39" t="n">
-        <v>2026-01-23</v>
+        <v>2026-12-14</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>A04FS</t>
+          <t>A17FS</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2235,81 +3022,60 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>AC4.3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HITO</t>
+          <t>ACTIVIDAD</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Diseño aprobado</t>
+          <t>Cierre del proyecto</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>AC21</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>2026-02-10</v>
-      </c>
-      <c r="F40" t="n">
-        <v>2026-02-10</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>A07FS</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>E4</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>H04</t>
+          <t>A19</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HITO</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Integración disponible</t>
+          <t>Evaluar resultados del piloto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>AC31</t>
+          <t>AC4.3</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2026-03-11</v>
+        <v>2026-12-15</v>
       </c>
       <c r="F41" t="n">
-        <v>2026-03-11</v>
+        <v>2026-12-17</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>A12FS</t>
+          <t>A18FS</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2321,38 +3087,38 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>H05</t>
+          <t>A20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>HITO</t>
+          <t>SUBACTIVIDAD</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>UAT aprobada</t>
+          <t>Elaborar informe y acta de cierre</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>AC33</t>
+          <t>AC4.3</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2026-03-27</v>
+        <v>2026-12-18</v>
       </c>
       <c r="F42" t="n">
-        <v>2026-03-27</v>
+        <v>2026-12-21</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>A15FS</t>
+          <t>A19FS</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2374,19 +3140,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Cierre formal aprobado</t>
+          <t>Cierre formal del proyecto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>AC43</t>
+          <t>AC4.3</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2026-04-23</v>
+        <v>2026-12-21</v>
       </c>
       <c r="F43" t="n">
-        <v>2026-04-23</v>
+        <v>2026-12-21</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2451,12 +3217,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>R001</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ana Analista</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2466,12 +3232,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Analista Funcional</t>
+          <t>Jefe de Proyecto</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>22000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2488,12 +3254,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R002</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bruno Backend</t>
+          <t>María Soto</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2503,12 +3269,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Desarrollador Backend</t>
+          <t>Analista Funcional / de Negocio</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>24000</t>
+          <t>22000</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2525,12 +3291,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R003</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Carla Frontend</t>
+          <t>Diego López</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2540,7 +3306,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Desarrollador Frontend/Móvil</t>
+          <t>Desarrollador Backend</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2562,12 +3328,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>R004</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Diego QA</t>
+          <t>Christian Pérez</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2577,12 +3343,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Analista QA</t>
+          <t>Desarrollador Frontend/Móvil</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>18500</t>
+          <t>24000</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2599,12 +3365,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>R005</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Elena Proyecto</t>
+          <t>Pedro Rivas</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2614,12 +3380,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Analista QA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>18500</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2636,12 +3402,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>R006</t>
+          <t>R-EQ1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kit tablets de obra</t>
+          <t>Tablets rugerizadas</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2651,12 +3417,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Dispositivo</t>
+          <t>Equipamiento</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>350000</t>
+          <t>480000</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2668,12 +3434,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>R007</t>
+          <t>R-IN1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nube de prueba</t>
+          <t>Infraestructura cloud QA y producción</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2683,12 +3449,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cloud</t>
+          <t>Infraestructura y licencias</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1200000</t>
+          <t>850000</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2700,12 +3466,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R008</t>
+          <t>R-SE1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Servicio API externo</t>
+          <t>Prueba de seguridad externa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2715,12 +3481,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Proveedor</t>
+          <t>Servicio externo</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3000000</t>
+          <t>2400000</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2776,12 +3542,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R001</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2793,39 +3559,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R002</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R003</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2837,171 +3603,171 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R004</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R005</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R001</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R002</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A08</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R003</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A09</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R004</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>R005</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>36</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>R001</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3013,17 +3779,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R002</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3035,17 +3801,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>A09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>R003</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>96</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3057,39 +3823,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>A10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>R004</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>A11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R005</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3101,17 +3867,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>A16</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R001</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3123,17 +3889,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>A17</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R002</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -3145,12 +3911,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>A18</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R003</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3160,100 +3926,293 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>A19</t>
+          <t>A14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R004</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>A20</t>
+          <t>A15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>R005</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>A15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R006</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2</t>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>A16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>R007</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>1</t>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>A17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>R008</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>A19</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>A19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>A20</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>A18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>R-EQ1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>R-IN1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>R-IN1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>R-SE1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3306,152 +4265,260 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Evidencia aprobada del hito 01</t>
+          <t>Acta de alcance firmada por el cliente</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Acta firmada y revisión del entregable</t>
+          <t>Revisión del entregable y del acta en comité</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>H02</t>
+          <t>H01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CR-H02-01</t>
+          <t>CR-H01-02</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Evidencia aprobada del hito 02</t>
+          <t>Backlog priorizado publicado</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Acta firmada y revisión del entregable</t>
+          <t>Revisión del entregable y del acta en comité</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CR-H03-01</t>
+          <t>CR-H02-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Evidencia aprobada del hito 03</t>
+          <t>Prototipo validado con 3 jefes de obra</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Acta firmada y revisión del entregable</t>
+          <t>Revisión del entregable y del acta en comité</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H04</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CR-H04-01</t>
+          <t>CR-H02-02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Evidencia aprobada del hito 04</t>
+          <t>Arquitectura aprobada por TI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Acta firmada y revisión del entregable</t>
+          <t>Revisión del entregable y del acta en comité</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>H05</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CR-H05-01</t>
+          <t>CR-H03-01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Evidencia aprobada del hito 05</t>
+          <t>API y app desplegadas en QA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Acta firmada y revisión del entregable</t>
+          <t>Revisión del entregable y del acta en comité</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Jefe de Proyecto</t>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>H03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CR-H03-02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Reportes exportan a PDF</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Revisión del entregable y del acta en comité</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Kevin Henríquez</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CR-H04-01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Acta UAT firmada</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Revisión del entregable y del acta en comité</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Kevin Henríquez</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CR-H04-02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0 defectos críticos abiertos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Revisión del entregable y del acta en comité</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Kevin Henríquez</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CR-H05-01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>App en producción en la obra piloto</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Revisión del entregable y del acta en comité</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kevin Henríquez</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>CR-H06-01</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Evidencia aprobada del hito 06</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Acta firmada y revisión del entregable</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Jefe de Proyecto</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Acta de cierre firmada por el patrocinador</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Revisión del entregable y del acta en comité</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Kevin Henríquez</t>
         </is>
       </c>
     </row>
@@ -3482,7 +4549,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>A04</t>
         </is>
       </c>
     </row>
@@ -3494,53 +4561,77 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>A05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>H03</t>
+          <t>H02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>A06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H04</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>A08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>H05</t>
+          <t>H03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>A10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>H04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>H05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>H06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>A20</t>
         </is>
@@ -3615,7 +4706,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -3627,7 +4718,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clasificación</t>
+          <t>Clasificación y prioridad</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3637,7 +4728,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -3659,7 +4750,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -3681,7 +4772,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -3703,7 +4794,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -3715,7 +4806,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Planificación</t>
+          <t>Planificación del cambio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3725,7 +4816,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -3747,7 +4838,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>120</t>
         </is>
       </c>
     </row>
@@ -3769,7 +4860,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -3781,7 +4872,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cierre</t>
+          <t>Cierre y línea base</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3791,7 +4882,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -3835,29 +4926,29 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>delta_dias</t>
+          <t>solicitante</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>delta_costo</t>
+          <t>justificacion</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CR-001</t>
+          <t>CB-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ajustar duración de integración</t>
+          <t>Agregar firma digital del inspector</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PLAZO</t>
+          <t>ALCANCE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -3877,29 +4968,24 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>480000</t>
+          <t>Jefe de obra Viña del Mar</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CR-002</t>
+          <t>CB-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Agregar tablet para piloto</t>
+          <t>Extender pruebas de sistema en 3 días</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RECURSOS</t>
+          <t>PLAZO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -3919,29 +5005,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>350000</t>
+          <t>Analista QA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CR-003</t>
+          <t>CB-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Incluir reporte ejecutivo</t>
+          <t>Comprar 2 tablets adicionales</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ALCANCE</t>
+          <t>COSTO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -3961,66 +5042,56 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>960000</t>
+          <t>Administración de obra</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CR-004</t>
+          <t>CB-04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cambiar proveedor API</t>
+          <t>Sumar apoyo QA en UAT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>COSTO</t>
+          <t>RECURSOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>APROBADA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Planificación del cambio</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>1200000</t>
+          <t>Jefe de Proyecto</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CR-005</t>
+          <t>CB-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cerrar capacitación piloto</t>
+          <t>Exportar reportes a Excel editable</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4030,27 +5101,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>BAJA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>APROBADA</t>
+          <t>RECHAZADA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Cierre</t>
+          <t>Revisión del comité</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>220000</t>
+          <t>Oficina técnica</t>
         </is>
       </c>
     </row>

</xml_diff>